<commit_message>
Hoja IVA/IRPF: actualizar precios de referencia (+25 €)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017RgC5vCZJXS9Md3YP5kjE5
</commit_message>
<xml_diff>
--- a/apartar-iva-irpf.xlsx
+++ b/apartar-iva-irpf.xlsx
@@ -1127,7 +1127,7 @@
         <v>37</v>
       </c>
       <c r="B14" s="14" t="n">
-        <v>350</v>
+        <v>375</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>38</v>
@@ -1138,7 +1138,7 @@
         <v>39</v>
       </c>
       <c r="B15" s="14" t="n">
-        <v>250</v>
+        <v>275</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1146,7 +1146,7 @@
         <v>40</v>
       </c>
       <c r="B16" s="14" t="n">
-        <v>550</v>
+        <v>575</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1154,7 +1154,7 @@
         <v>41</v>
       </c>
       <c r="B17" s="14" t="n">
-        <v>150</v>
+        <v>175</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1162,7 +1162,7 @@
         <v>42</v>
       </c>
       <c r="B18" s="14" t="n">
-        <v>550</v>
+        <v>575</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>